<commit_message>
Campanhas, foto com legenda e respostas por número
- Menu por campanhas (planilha + mensagem + regras)
- Mensagem com imagem enviada como foto com legenda (nunca figurinha)
- Nome na mensagem, detecção de cabeçalho/colunas e coluna de controle Não/Sim
- Todas as respostas com 1/2/0; aviso quando a planilha não existe
- README, docs, planilha e imagem de exemplo atualizados

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados/contatos-exemplo.xlsx
+++ b/dados/contatos-exemplo.xlsx
@@ -413,18 +413,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Nome completo</t>
+          <t>Nome</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Nome</t>
+          <t>Telefone</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
@@ -434,19 +434,19 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Telefone</t>
+          <t>Mensagem enviada?</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>maria silva souza</t>
+          <t>MARIA SILVA</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Maria</t>
+          <t>15991234567</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -456,19 +456,19 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>15991234567</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>joão pedro lima</t>
+          <t>joão pedro</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>João</t>
+          <t>11987654321</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -478,19 +478,19 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11987654321</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ana costa</t>
+          <t>Ana</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Ana</t>
+          <t>1698765432</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -500,19 +500,19 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1698765432</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>carlos eduardo dias</t>
+          <t>Carlos</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>13055550123</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -522,7 +522,29 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>13055550123</t>
+          <t>Não</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Beatriz Costa</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>21988887777</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>bia@exemplo.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Não</t>
         </is>
       </c>
     </row>

</xml_diff>